<commit_message>
Site-wide plain-voice pass: no em dashes, no GRE words
Applies the teaching-page style rules everywhere: home, projects,
writing, selected work, dashboard, data dictionary, and both
interactive templates. Em dashes become commas, colons, parentheses,
or sentence breaks; fancy words get plain ones (methodological,
doctrinal, utilization, operationalization, non-Anglophone,
provisional, uncannily, synthesis...).

Also fixes 28 em-dash cells inside the two Excel workbooks (artist
descriptions, confidence notes, Data Dictionary sheet, Barnum
statements) via exact-match cell replacement, and updates the
teaching page's artist count to the expanded 163-act dataset.
Freeze caches for the dashboard and data dictionary were rebuilt so
the rendered tables pick up the new workbook text.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/barnum/data/barnum_statements.xlsx
+++ b/barnum/data/barnum_statements.xlsx
@@ -1,23 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="" yWindow="" windowWidth="" windowHeight="" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Statements" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Research" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Distribution" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t xml:space="preserve">Self-criticism is almost universal, especially among the kind of person who would sit down to take a personality test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Appeals to your self-image as a critical thinker. Ironic, given you are being asked to accept this very statement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most people both value some routine and dislike too much of it, so this fits nearly anyone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-flattering and nearly universal: almost everyone feels under-appreciated some of the time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decades of replications cluster around a mean accuracy of roughly 4.0-4.3 out of 5; the effect is one of the most reliably reproduced in psychology.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
   <fonts count="2">
     <font>
@@ -28,13 +47,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <sz val="11"/>
       <color rgb="00FFFFFF"/>
+      <name val="Calibri"/>
+      <b/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -58,14 +79,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -422,18 +444,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="5" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="64" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="70" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,10 +514,8 @@
           <t>Universal validation</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Self-criticism is almost universal — especially among the kind of person who would sit down to take a personality test.</t>
-        </is>
+      <c r="D3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -572,10 +592,8 @@
           <t>Flattery</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Appeals to your self-image as a critical thinker — ironic, given you are being asked to accept this very statement.</t>
-        </is>
+      <c r="D7" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -672,10 +690,8 @@
           <t>Double-headed</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Most people both value some routine and dislike too much of it — so this fits nearly anyone.</t>
-        </is>
+      <c r="D12" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -752,10 +768,8 @@
           <t>Flattery</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Self-flattering and near-universal — almost everyone feels under-appreciated some of the time.</t>
-        </is>
+      <c r="D16" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -780,25 +794,26 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="8" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="60" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="60" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -873,8 +888,8 @@
           <t>Typical replication range</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="B3"/>
+      <c r="C3"/>
       <c r="D3" t="n">
         <v>5</v>
       </c>
@@ -886,28 +901,27 @@
           <t>Summary of subsequent replications across decades (see, e.g., reviews of the Barnum/Forer effect).</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Decades of replications cluster around a mean accuracy of roughly 4.0-4.3 out of 5 — the effect is one of the most reliably reproduced in psychology.</t>
-        </is>
+      <c r="G3" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1012,5 +1026,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>